<commit_message>
ORFS: swivels at every size, counterbore-mouth masters, straight swivel reference settled
- fsmeasure: counterbore mouth, no-lip neck, nut rear face below the stem head (pilots 0 FAIL)
- gen_tee: FSSW_MEAS -04 ... -20 from FS6500-NN (fssw_table, -08 identical), counterbore mouth
  (-10 up), nut-wall check at the relief; masters per leg shape step / neck / mouth
- FS6565-08-08: Air-Way's straight swivel length runs to the stem seal face
- 101 FS configurations: static checks clean, OCP closed loops 2,636 checks 0 off,
  regression 99 / 99 identical (regress_all now lists derived roots too)
- count 1,517 of 2,535 ready after SolidWorks; README step 5, status, hand-over

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QQuceHR8ZUuy6411Z8yX1P
</commit_message>
<xml_diff>
--- a/tools/_out/orfs_gen_20261020/out/tee/DesignTable_FS2500N_SW2.xlsx
+++ b/tools/_out/orfs_gen_20261020/out/tee/DesignTable_FS2500N_SW2.xlsx
@@ -788,7 +788,7 @@
       </c>
       <c r="AP2" t="inlineStr">
         <is>
-          <t>ORFS 90 deg Elbow (male face seal x male face seal) - face-seal legs without a step (flats = thread), 9/16-18 UN (male O-ring face seal, SAE J1453) x 9/16-18 UN (male O-ring face seal, SAE J1453)</t>
+          <t>ORFS 90 deg Elbow (male face seal x male face seal) - face-seal legs with the flats = the thread major (no step), 9/16-18 UN (male O-ring face seal, SAE J1453) x 9/16-18 UN (male O-ring face seal, SAE J1453)</t>
         </is>
       </c>
       <c r="AQ2" t="inlineStr">
@@ -957,7 +957,7 @@
       </c>
       <c r="AP3" t="inlineStr">
         <is>
-          <t>ORFS 90 deg Elbow (male face seal x male face seal) - face-seal legs without a step (flats = thread), 1 3/16-12 UN (male O-ring face seal, SAE J1453) x 1 3/16-12 UN (male O-ring face seal, SAE J1453)</t>
+          <t>ORFS 90 deg Elbow (male face seal x male face seal) - face-seal legs with the flats = the thread major (no step), 1 3/16-12 UN (male O-ring face seal, SAE J1453) x 1 3/16-12 UN (male O-ring face seal, SAE J1453)</t>
         </is>
       </c>
       <c r="AQ3" t="inlineStr">
@@ -1126,7 +1126,7 @@
       </c>
       <c r="AP4" t="inlineStr">
         <is>
-          <t>ORFS 90 deg Elbow (male face seal x male face seal) - face-seal legs without a step (flats = thread), 1 7/16-12 UN (male O-ring face seal, SAE J1453) x 1 7/16-12 UN (male O-ring face seal, SAE J1453)</t>
+          <t>ORFS 90 deg Elbow (male face seal x male face seal) - face-seal legs with the flats = the thread major (no step), 1 7/16-12 UN (male O-ring face seal, SAE J1453) x 1 7/16-12 UN (male O-ring face seal, SAE J1453)</t>
         </is>
       </c>
       <c r="AQ4" t="inlineStr">

</xml_diff>